<commit_message>
chore: publish document IG 2.0.1
</commit_message>
<xml_diff>
--- a/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
+++ b/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
   <si>
     <t>Property</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0</t>
+    <t>2.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -67,7 +67,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-01</t>
+    <t>2026-03-10</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -127,7 +127,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>32</t>
+    <t>33</t>
   </si>
   <si>
     <t>Code</t>
@@ -323,6 +323,12 @@
   </si>
   <si>
     <t>DK EKG schema</t>
+  </si>
+  <si>
+    <t>urn:ad:dk:medcom:ecn-v1.0:full</t>
+  </si>
+  <si>
+    <t>DK ECN schema</t>
   </si>
 </sst>
 </file>
@@ -678,7 +684,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1079,6 +1085,18 @@
       </c>
       <c r="D33" s="2"/>
     </row>
+    <row r="34">
+      <c r="A34" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="B34" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="C34" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="D34" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: publish document IG 2.0.1 (#71)
Co-authored-by: tmsMedcom <tmsMedcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
+++ b/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
   <si>
     <t>Property</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0</t>
+    <t>2.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -67,7 +67,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-01</t>
+    <t>2026-03-10</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -127,7 +127,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>32</t>
+    <t>33</t>
   </si>
   <si>
     <t>Code</t>
@@ -323,6 +323,12 @@
   </si>
   <si>
     <t>DK EKG schema</t>
+  </si>
+  <si>
+    <t>urn:ad:dk:medcom:ecn-v1.0:full</t>
+  </si>
+  <si>
+    <t>DK ECN schema</t>
   </si>
 </sst>
 </file>
@@ -678,7 +684,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1079,6 +1085,18 @@
       </c>
       <c r="D33" s="2"/>
     </row>
+    <row r="34">
+      <c r="A34" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="B34" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="C34" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="D34" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: publish document IG 2.0.2
</commit_message>
<xml_diff>
--- a/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
+++ b/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="106">
   <si>
     <t>Property</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.1</t>
+    <t>2.0.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -67,7 +67,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-10</t>
+    <t>2026-04-28</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -127,7 +127,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>33</t>
+    <t>34</t>
   </si>
   <si>
     <t>Code</t>
@@ -329,6 +329,9 @@
   </si>
   <si>
     <t>DK ECN schema</t>
+  </si>
+  <si>
+    <t>urn:ad:dk:medcom:ekg-v2.0:full</t>
   </si>
 </sst>
 </file>
@@ -684,7 +687,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1097,6 +1100,18 @@
       </c>
       <c r="D34" s="2"/>
     </row>
+    <row r="35">
+      <c r="A35" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="B35" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="C35" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="D35" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: publish document IG 2.0.2 (#75)
Co-authored-by: RikkeVestesen <RikkeVestesen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
+++ b/ig/document/CodeSystem-MedCom-ihe-formatcode-CS-TEMP.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="106">
   <si>
     <t>Property</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.1</t>
+    <t>2.0.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -67,7 +67,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-10</t>
+    <t>2026-04-28</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -127,7 +127,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>33</t>
+    <t>34</t>
   </si>
   <si>
     <t>Code</t>
@@ -329,6 +329,9 @@
   </si>
   <si>
     <t>DK ECN schema</t>
+  </si>
+  <si>
+    <t>urn:ad:dk:medcom:ekg-v2.0:full</t>
   </si>
 </sst>
 </file>
@@ -684,7 +687,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1097,6 +1100,18 @@
       </c>
       <c r="D34" s="2"/>
     </row>
+    <row r="35">
+      <c r="A35" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="B35" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="C35" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="D35" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>